<commit_message>
Update logbook from 20260113
</commit_message>
<xml_diff>
--- a/data/microCTD/20260113/Level0/Logbook_Zug_20260112.xlsx
+++ b/data/microCTD/20260113/Level0/Logbook_Zug_20260112.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unils-my.sharepoint.com/personal/tomy_doda_unil_ch/Documents/Projects-GSE42572/3-Zug/turbulence-lakezug/data/microCTD/20260113/Level0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="626" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6F289ED-7788-4768-BF55-8B19D6F4E3AA}"/>
+  <xr:revisionPtr revIDLastSave="627" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48484060-9814-4050-910A-121C1BE3DDF0}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="3480" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Logbook_Zug" sheetId="1" r:id="rId1"/>
@@ -1644,7 +1644,7 @@
       <c r="K13" s="40"/>
       <c r="L13" s="40"/>
       <c r="M13" s="40">
-        <v>380136</v>
+        <v>680136</v>
       </c>
       <c r="N13" s="40">
         <v>218745</v>

</xml_diff>

<commit_message>
Modify logbook from 20260113: replace VMPC by VMPW for western profiles
</commit_message>
<xml_diff>
--- a/data/microCTD/20260113/Level0/Logbook_Zug_20260112.xlsx
+++ b/data/microCTD/20260113/Level0/Logbook_Zug_20260112.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unils-my.sharepoint.com/personal/tomy_doda_unil_ch/Documents/Projects-GSE42572/3-Zug/turbulence-lakezug/data/microCTD/20260113/Level0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="627" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48484060-9814-4050-910A-121C1BE3DDF0}"/>
+  <xr:revisionPtr revIDLastSave="630" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1D737EC-98C2-4CAC-BEB2-881AA23D9A1D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Logbook_Zug" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
   <si>
     <t>Date</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t xml:space="preserve">Lake depth: 176 m. Drifting towards North. </t>
+  </si>
+  <si>
+    <t>VMPW</t>
   </si>
 </sst>
 </file>
@@ -768,31 +771,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA23"/>
-  <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="17.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="10.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.1796875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="10" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="10" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="5" customWidth="1"/>
-    <col min="10" max="11" width="14.5703125" style="5" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="10.85546875" style="4" customWidth="1"/>
-    <col min="14" max="14" width="7.7109375" style="4" customWidth="1"/>
-    <col min="15" max="18" width="17.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" style="10" customWidth="1"/>
+    <col min="8" max="8" width="20.54296875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" style="5" customWidth="1"/>
+    <col min="10" max="11" width="14.54296875" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="10.81640625" style="4" customWidth="1"/>
+    <col min="14" max="14" width="7.7265625" style="4" customWidth="1"/>
+    <col min="15" max="18" width="17.7265625" style="2" customWidth="1"/>
     <col min="19" max="19" width="11" style="2" customWidth="1"/>
-    <col min="20" max="20" width="11.85546875" style="2" customWidth="1"/>
-    <col min="21" max="21" width="9.28515625" style="2" customWidth="1"/>
-    <col min="22" max="23" width="9.42578125" style="2" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="2" customWidth="1"/>
+    <col min="20" max="20" width="11.81640625" style="2" customWidth="1"/>
+    <col min="21" max="21" width="9.26953125" style="2" customWidth="1"/>
+    <col min="22" max="23" width="9.453125" style="2" customWidth="1"/>
+    <col min="24" max="24" width="9.26953125" style="2" customWidth="1"/>
     <col min="25" max="25" width="14" style="2" customWidth="1"/>
-    <col min="26" max="26" width="91.42578125" style="5" customWidth="1"/>
+    <col min="26" max="26" width="91.453125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>2</v>
       </c>
@@ -872,7 +875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="19" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" s="19" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
         <v>24</v>
       </c>
@@ -951,7 +954,7 @@
       </c>
       <c r="AA2" s="31"/>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A3" s="23" t="s">
         <v>31</v>
       </c>
@@ -1017,7 +1020,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
         <v>31</v>
       </c>
@@ -1083,7 +1086,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A5" s="23" t="s">
         <v>31</v>
       </c>
@@ -1149,7 +1152,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:27" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>34</v>
       </c>
@@ -1216,7 +1219,7 @@
       </c>
       <c r="AA6"/>
     </row>
-    <row r="7" spans="1:27" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>34</v>
       </c>
@@ -1283,7 +1286,7 @@
       </c>
       <c r="AA7"/>
     </row>
-    <row r="8" spans="1:27" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
         <v>34</v>
       </c>
@@ -1350,7 +1353,7 @@
       </c>
       <c r="AA8"/>
     </row>
-    <row r="9" spans="1:27" s="36" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" s="36" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="32" t="s">
         <v>42</v>
       </c>
@@ -1386,7 +1389,7 @@
         <v>218604</v>
       </c>
       <c r="O9" s="32" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="P9" s="32">
         <v>90</v>
@@ -1416,7 +1419,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:27" s="36" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" s="36" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="32" t="s">
         <v>42</v>
       </c>
@@ -1452,7 +1455,7 @@
         <v>218615</v>
       </c>
       <c r="O10" s="32" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="P10" s="32">
         <v>95</v>
@@ -1482,7 +1485,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:27" s="36" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" s="36" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="32" t="s">
         <v>42</v>
       </c>
@@ -1518,7 +1521,7 @@
         <v>218623</v>
       </c>
       <c r="O11" s="32" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="P11" s="32">
         <v>100</v>
@@ -1548,7 +1551,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:27" s="42" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" s="42" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="38" t="s">
         <v>46</v>
       </c>
@@ -1614,7 +1617,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:27" s="42" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" s="42" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="38" t="s">
         <v>46</v>
       </c>
@@ -1680,25 +1683,25 @@
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.35">
       <c r="E14" s="29"/>
       <c r="F14" s="29"/>
       <c r="G14" s="29"/>
       <c r="H14" s="29"/>
       <c r="Z14" s="30"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.35">
       <c r="E15" s="29"/>
       <c r="F15" s="29"/>
       <c r="G15" s="29"/>
       <c r="H15" s="29"/>
       <c r="Z15" s="30"/>
     </row>
-    <row r="19" spans="5:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="5:12" x14ac:dyDescent="0.35">
       <c r="K19" s="20"/>
       <c r="L19" s="20"/>
     </row>
-    <row r="23" spans="5:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="5:12" x14ac:dyDescent="0.35">
       <c r="E23" s="22"/>
     </row>
   </sheetData>

</xml_diff>